<commit_message>
Add Arabic To_check and check_answ columns (To_chk_AR, Answ_AR)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JAu1NnEtyFdpjqezLDmDLJ
</commit_message>
<xml_diff>
--- a/checking_Mefraq_answers.xlsx
+++ b/checking_Mefraq_answers.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Answers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Answers'!$A$1:$N$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Answers'!$A$1:$P$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -72,11 +72,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -452,23 +455,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:P70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="80" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -519,25 +524,35 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>To_chk_AR</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>check_answ</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Answ_AR</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Ask_Oper</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>P_Zone_new</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>P_zone_ver</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>P_Zone_change</t>
         </is>
@@ -583,25 +598,35 @@
           <t>CHECK the pressure zone - if K140 or Safawi ? are theses two facilities connected ?</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>التحقق من منطقة الضغط: K140 أم الصفاوي؟ هل المنشأتان متصلتان؟</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>K140_PS (not Safawi). K140 PS lies inside this zone, Safawi PS ~25 km away. Area tapped DN100/63 on DN400 main from wells K136+K140 (YWC src: wells 136+140, Safawi WS) - same system, pressure from K140 side.</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>K140_PS وليس الصفاوي. محطة K140 داخل المنطقة والصفاوي تبعد 25 كم. المنطقة من خط DN400 من آبار 136+140 (نفس النظام)</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>K140_PS</t>
         </is>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="O2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -647,25 +672,35 @@
           <t>TO CHECK IF FROM Beshryyeh PS or Dir Al kahf PS ?</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة البشرية أم محطة دير الكهف؟</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Beshryyeh PS - keep Bishiryyah_PS. Field: DN200 from Beshryyeh PS (main filling Dir Al-Kahf tank). Dir Al-Kahf PS sits in this zone (990-1067m) but its pumps H=250m serve upper villages (id75). YWC names Dair Al Kahef PS</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>محطة البشرية - يبقى Bishiryyah_PS. خط DN200 من البشرية يغذي خزان دير الكهف، ومضخات دير الكهف للقرى الأعلى. تأكيد</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>Bishiryyah_PS</t>
         </is>
       </c>
-      <c r="M3" s="2" t="n">
+      <c r="O3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -707,25 +742,35 @@
           <t>Check if the resv Dair Al Qenn is used ? or bypassed ? if used how ?</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>هل خزان دير القن مستخدم أم يتم تجاوزه؟ وإذا مستخدم كيف؟</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Dair Al Qenn Resv NOT used - bypassed (Master plan: Dir Al-Qun Resv = Abandoned). Fed directly by DN150 from Dir Al-Kahf PS (YWC confirms). YWC has 2 schedules: Tal Rmah / Deir Al Qen+Jadaa+Mathnah+Mansoora</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>خزان دير القن غير مستخدم (مهجور بالمخطط الشمولي). تغذية مباشرة DN150 من محطة دير الكهف. يُقترح تقسيم تل الرماح عن الباقي</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Dir Al-kahf PS</t>
         </is>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="O4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -767,25 +812,35 @@
           <t>How many discharge lines ? split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>كم عدد خطوط الدفع؟ تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Koum Ahmar PS has 2 pumps (50m3/h@250m, 100m3/h@100m) and 2 distribution outlets DN125 + DN100 (field notes). This zone fed by DN125 (+DN100) -&gt; Koum Ahmar_PS_125. Confirm which pump feeds which line.</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>لمحطة الكوم الأحمر خطا توزيع DN125 وDN100. هذه المنطقة على DN125 ← Koum Ahmar_PS_125 - تأكيد</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>Koum Ahmar_PS_125</t>
         </is>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="O5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -831,25 +886,35 @@
           <t>How many discharge lines ? split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>كم عدد خطوط الدفع؟ تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Koum Ahmar PS has 2 pumps (50m3/h@250m, 100m3/h@100m) and 2 distribution outlets DN125 + DN100 (field notes). This zone fed by DN100 -&gt; Koum Ahmar_PS_100. Confirm which pump feeds which line.</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>لمحطة الكوم الأحمر خطا توزيع DN125 وDN100. هذه المنطقة على DN100 ← Koum Ahmar_PS_100 - تأكيد مع المشغل</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Koum Ahmar_PS_100</t>
         </is>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="O6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -895,25 +960,35 @@
           <t>How many discharge lines ? split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>كم عدد خطوط الدفع؟ تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Koum Ahmar PS has 2 pumps (50m3/h@250m, 100m3/h@100m) and 2 distribution outlets DN125 + DN100 (field notes). This zone fed by DN100 -&gt; Koum Ahmar_PS_100. Confirm which pump feeds which line.</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>لمحطة الكوم الأحمر خطا توزيع DN125 وDN100. هذه المنطقة على DN100 ← Koum Ahmar_PS_100 - تأكيد مع المشغل</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>Koum Ahmar_PS_100</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="O7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -959,25 +1034,35 @@
           <t>How many discharge lines ? split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>كم عدد خطوط الدفع؟ تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Koum Ahmar PS has 2 pumps (50m3/h@250m, 100m3/h@100m) and 2 distribution outlets DN125 + DN100 (field notes). Zone fed by DN100 (+DN50) -&gt; Koum Ahmar_PS_100. GIS network differs - update.</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>لمحطة الكوم الأحمر خطا توزيع DN125 وDN100. المنطقة على DN100 (+DN50) ← Koum Ahmar_PS_100. تحديث GIS</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>Koum Ahmar_PS_100</t>
         </is>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="O8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1023,25 +1108,35 @@
           <t>Check if really they by-pass the reservoir of Bweidha</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً يتم تجاوز خزان البويضة</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>NO bypass here: fed by DN100 DISCHARGE from Bweidha PS (field notes), YWC: BWAIDAH PS. Change P_Zone to Bweidha_PS_100.</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>لا يوجد تجاوز: التغذية بخط دفع DN100 من محطة البويضة. تغيير إلى Bweidha_PS_100</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>Bweidha_PS_100</t>
         </is>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="O9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1087,25 +1182,35 @@
           <t>Check if really they by-pass the reservoir of Bweidha</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً يتم تجاوز خزان البويضة</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Yes - bypass confirmed: DN150 tapped on DN300 bypassing Bweidha Resv (1 bar) + DN100 from Bweidha PS discharge (double feed). YWC: UM LOLO PS (DN300 = Um Lulu PS water). Keep BYPASS.</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>نعم تجاوز جزئي: DN150 من خط DN300 متجاوز خزان البويضة + DN100 من دفع المحطة (تغذية مزدوجة). يبقى BYPASS - تأكيد</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>Bweidha_Resv_BYPASS</t>
         </is>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="O10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1147,25 +1252,35 @@
           <t>Check if really they by-pass the reservoir of Bweidha</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً يتم تجاوز خزان البويضة</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Yes - bypass confirmed: fed by DN300 bypassing Bweidha Resv (residual 1 bar). YWC source = UM LOLO PS, i.e. water comes directly from Um Lulu PS through DN300. Keep Bweidha_Resv_BYPASS.</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>نعم تجاوز مؤكد: من خط DN300 متجاوز خزان البويضة (ضغط 1 بار). YWC: محطة أم اللولو أي المياه مباشرة منها. يبقى BYPASS</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>Bweidha_Resv_BYPASS</t>
         </is>
       </c>
-      <c r="M11" s="2" t="n">
+      <c r="O11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1207,25 +1322,35 @@
           <t>Check if really they by-pass the reservoir of Bweidha</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً يتم تجاوز خزان البويضة</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Yes - bypass confirmed: fed by DN300 bypassing Bweidha Resv (residual 1 bar). YWC source = UM LOLO PS, i.e. water comes directly from Um Lulu PS through DN300. Keep Bweidha_Resv_BYPASS.</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>نعم تجاوز مؤكد: من خط DN300 متجاوز خزان البويضة (ضغط 1 بار). YWC: محطة أم اللولو أي المياه مباشرة منها. يبقى BYPASS</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>Bweidha_Resv_BYPASS</t>
         </is>
       </c>
-      <c r="M12" s="2" t="n">
+      <c r="O12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1267,25 +1392,35 @@
           <t>Check if really they by-pass the reservoir of Bweidha</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً يتم تجاوز خزان البويضة</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Yes - bypass confirmed: 2 x DN200 taps on DN300 bypassing Bweidha Resv (1 bar), 12 valves split zone 6-8h each. YWC: BWAIDAH PS. Keep Bweidha_Resv_BYPASS.</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>نعم تجاوز مؤكد: 2×DN200 من خط DN300 (1 بار)، 12 محبس 6-8 ساعات لكل منطقة. يبقى Bweidha_Resv_BYPASS</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>Bweidha_Resv_BYPASS</t>
         </is>
       </c>
-      <c r="M13" s="2" t="n">
+      <c r="O13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1327,25 +1462,35 @@
           <t>Check if really they by-pass the reservoir of Bweidha</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً يتم تجاوز خزان البويضة</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Yes - bypass confirmed: DN100 tapped on DN300 bypassing Bweidha Resv, but this line is OUT OF SERVICE (field). Qadam Resv = Abandoned (MP). Ask operator current supply.</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>نعم تجاوز: DN100 من خط DN300 لكنه متوقف، وخزان القدم مهجور. اسأل المشغل عن مصدر التغذية الحالي</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>Bweidha_Resv_BYPASS</t>
         </is>
       </c>
-      <c r="M14" s="2" t="n">
+      <c r="O14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1387,25 +1532,35 @@
           <t>Check if really they by-pass the reservoir of Bweidha</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً يتم تجاوز خزان البويضة</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Yes - bypass confirmed: DN200 branch next to Qadam Resv; Qadam Resv is Abandoned (MP) so the line is not re-stored. YWC: BWAIDAH PS. Keep BYPASS; update GIS: DN200 Qadam-&gt;Maamaria.</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>نعم تجاوز: فرع DN200 بجانب خزان القدم (مهجور). يبقى BYPASS. تحديث GIS: خط DN200 من القدم للمعمرية</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>Bweidha_Resv_BYPASS</t>
         </is>
       </c>
-      <c r="M15" s="2" t="n">
+      <c r="O15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1447,25 +1602,35 @@
           <t>Check if really they by-pass the reservoir of Bweidha</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً يتم تجاوز خزان البويضة</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Yes - bypass confirmed: DN200 branch next to Qadam Resv; Qadam Resv is Abandoned (MP) so the line is not re-stored. YWC: BWAIDAH PS. Keep BYPASS; update GIS: DN200 Qadam-&gt;Maamaria.</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>نعم تجاوز: فرع DN200 بجانب خزان القدم (مهجور). يبقى BYPASS. تحديث GIS: خط DN200 من القدم للمعمرية</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>Bweidha_Resv_BYPASS</t>
         </is>
       </c>
-      <c r="M16" s="2" t="n">
+      <c r="O16" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1507,25 +1672,35 @@
           <t>Check from where it's fed Bwaida_Reservoir_300_gravity or Rehab_Resv ?</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>التحقق من مصدر التغذية: خط البويضة 300 بالانسياب أم خزان رحاب؟</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Fed from Bweidha DN300 (DN150 tapped on DN300, no connections on DN150) - NOT Rehab: Rhab PS is 60m3/h@300m booster with 25m3 tank. YWC: BWAIDAH PS. Keep Bweidha_Resv_300_G.</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>من خط البويضة DN300 (فرع DN150) وليس خزان رحاب؛ رحاب محطة تقوية صغيرة. يبقى Bweidha_Resv_300_G</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>Bweidha_Resv_300_G</t>
         </is>
       </c>
-      <c r="M17" s="2" t="n">
+      <c r="O17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1567,25 +1742,35 @@
           <t>Check from where it's fed Bwaida_Reservoir_300_gravity or Rehab_Resv ?</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>التحقق من مصدر التغذية: خط البويضة 300 بالانسياب أم خزان رحاب؟</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Fed from Bweidha DN300 (DN150 tapped on DN300, no connections on DN150) - NOT Rehab: Rhab PS is 60m3/h@300m booster with 25m3 tank. YWC: BWAIDAH PS. Keep Bweidha_Resv_300_G.</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>من خط البويضة DN300 (فرع DN150) وليس خزان رحاب؛ رحاب محطة تقوية صغيرة. يبقى Bweidha_Resv_300_G</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>Bweidha_Resv_300_G</t>
         </is>
       </c>
-      <c r="M18" s="2" t="n">
+      <c r="O18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1627,25 +1812,35 @@
           <t>Check from where it's fed Bwaida_Reservoir_300_gravity or Rehab_Resv ?</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>التحقق من مصدر التغذية: خط البويضة 300 بالانسياب أم خزان رحاب؟</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Fed from Bweidha DN300 (DN150 tapped on DN300, no connections on DN150) - NOT Rehab: Rhab PS is 60m3/h@300m booster with 25m3 tank. YWC: BWAIDAH PS. Keep Bweidha_Resv_300_G (DN125 on DN150).</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>من خط البويضة DN300 (فرع DN150) وليس خزان رحاب؛ رحاب محطة تقوية صغيرة. يبقى Bweidha_Resv_300_G</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>Bweidha_Resv_300_G</t>
         </is>
       </c>
-      <c r="M19" s="2" t="n">
+      <c r="O19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1687,25 +1882,35 @@
           <t>Check if fed from Dogmseh_PS or Bweida_PS</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة الدقمسة أم محطة البويضة</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS. YWC: DOGMOSEH PS. Dogmseh PS (2 pumps 50m3/h@400m/@250m, 4x25m3 tanks) is fed from Bweidha system; zone boosted by Dogmseh PS 4h for high points (DN125 from DN150). Keep Dogmseh_PS.</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>محطة الدقمسة (YWC). تقوية 4 ساعات للمرتفعات والمياه أصلاً من نظام البويضة. يبقى Dogmseh_PS</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS</t>
         </is>
       </c>
-      <c r="M20" s="2" t="n">
+      <c r="O20" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1747,25 +1952,35 @@
           <t>Check if fed from Dogmseh_PS or Bweida_PS</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة الدقمسة أم محطة البويضة</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS. YWC: DOGMOSEH PS. Dogmseh PS (2 pumps 50m3/h@400m/@250m, 4x25m3 tanks) is fed from Bweidha system; zone boosted by Dogmseh PS 4h for high points (DN100 from DN150). Keep Dogmseh_PS.</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>محطة الدقمسة (YWC). تقوية 4 ساعات للمرتفعات والمياه أصلاً من نظام البويضة. يبقى Dogmseh_PS</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS</t>
         </is>
       </c>
-      <c r="M21" s="2" t="n">
+      <c r="O21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1807,25 +2022,35 @@
           <t>Check from where it's fed Bwaida_Reservoir_300_gravity or Rehab_Resv ?</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>التحقق من مصدر التغذية: خط البويضة 300 بالانسياب أم خزان رحاب؟</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Neither Bweidha nor Rehab: YWC lists MEDWAR under QNAYYA PS (Qnayya WS). Nearest zones Khatla/Dahal = Al-Qnaya_PS DN150-&gt;DN100, field: DN100 continues south. Change to Al-Qnaya_PS - confirm.</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>لا البويضة ولا رحاب: YWC يضع المدور على محطة القنية. تغيير إلى Al-Qnaya_PS - تأكيد</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>Al-Qnaya_PS</t>
         </is>
       </c>
-      <c r="M22" s="2" t="n">
+      <c r="O22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N22" s="2" t="inlineStr">
+      <c r="P22" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1871,25 +2096,35 @@
           <t>Check if fed from Zaatary_PS or Sumaya_PS or Hayan_booster</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة الزعتري أم محطة سمية أم بوستر حيان</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>Zaatary_PS_400 (confirmed). DN200 tapped on Zaatari DN400 discharge next to Hayyan PS. YWC: HAYYAN BOOSTER/ZAATARI PS - booster is downstream on same line; zone takes Zaatari DN400 pressure.</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr">
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Zaatary_PS_400 مؤكد: فرع من خط دفع الزعتري DN400 قرب بوستر حيان، والضغط من الزعتري</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr">
         <is>
           <t>Zaatary_PS_400</t>
         </is>
       </c>
-      <c r="M23" s="2" t="n">
+      <c r="O23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1931,25 +2166,35 @@
           <t>Check if fed from Zaatary_PS or Sumaya_PS or Hayan_booster</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة الزعتري أم محطة سمية أم بوستر حيان</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>Zaatary_PS_400 (confirmed). DN100 + direct connections on Zaatari DN400 discharge before Hayyan PS. YWC: HAYYAN BOOSTER/ZAATARI PS - zone takes Zaatari DN400 pressure.</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>Zaatary_PS_400 مؤكد: فرع من خط دفع الزعتري DN400 قرب بوستر حيان، والضغط من الزعتري</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>Zaatary_PS_400</t>
         </is>
       </c>
-      <c r="M24" s="2" t="n">
+      <c r="O24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1991,25 +2236,35 @@
           <t>is this area fed by the Reservoir Hudud or by Jaber PS ?</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>هل تتغذى المنطقة من خزان الحدود أم من محطة جابر؟</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>Hudud Reservoir (gravity). Reservoir lies inside this zone and is filled by DN100 from Jaber PS; network fed from Resv (field). YWC: HODOOD RES. Keep Jaber_Resv (better: Hudud_Jaber_Resv). MP: access needs permit.</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>خزان الحدود بالانسياب؛ الخزان داخل المنطقة ويُعبأ بخط DN100 من محطة جابر. يبقى Jaber_Resv</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="N25" s="2" t="inlineStr">
         <is>
           <t>Jaber_Resv</t>
         </is>
       </c>
-      <c r="M25" s="2" t="n">
+      <c r="O25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2051,25 +2306,35 @@
           <t>Check if fe from Sumaya_PS or Hayyan_Booster ?</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة سمية أم بوستر حيان؟</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Sumaya PS (not Hayyan booster). YWC: SUMAYYA PS; field notes: direct from Sumaya DN400 line -&gt; DN200 -&gt; DN150 branches. Hayyan booster is 20 m away but not feeding. Keep Sumaya PS_400.</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>محطة سمية وليس بوستر حيان (YWC + خط DN400 مباشر من سمية). يبقى Sumaya PS_400</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>Sumaya PS_400</t>
         </is>
       </c>
-      <c r="M26" s="2" t="n">
+      <c r="O26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2111,25 +2376,35 @@
           <t>Check if fe from Sumaya_PS or Hayyan_Booster ?</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة سمية أم بوستر حيان؟</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>Sumaya PS (not Hayyan booster). YWC: SUMAYYA PS; field notes: direct from Sumaya DN400 line (DN400/500) -&gt; DN150/125 branches. Keep Sumaya PS_400.</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>محطة سمية وليس بوستر حيان (YWC + خط DN400 مباشر من سمية). يبقى Sumaya PS_400</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
         <is>
           <t>Sumaya PS_400</t>
         </is>
       </c>
-      <c r="M27" s="2" t="n">
+      <c r="O27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2171,25 +2446,35 @@
           <t>Check if fed from Sumaya_PS or Hayyan_Booster ?</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة سمية أم بوستر حيان؟</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>Sumaya PS (not Hayyan booster). YWC: SUMAYYA PS; field notes: direct from Sumaya DN400 line (DN400/500) -&gt; DN150/125 branches. Hayyan booster is next to zone but not feeding. Keep Sumaya PS_400.</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>محطة سمية وليس بوستر حيان (YWC + خط DN400 مباشر من سمية). يبقى Sumaya PS_400</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>Sumaya PS_400</t>
         </is>
       </c>
-      <c r="M28" s="2" t="n">
+      <c r="O28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -2231,25 +2516,35 @@
           <t>Check if fe from Sumaya_PS or Hayyan_Booster ?</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة سمية أم بوستر حيان؟</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>Sumaya PS (not Hayyan booster). YWC: SUMAYYA PS; field notes: direct from Sumaya DN400 line reduced to DN200 -&gt; DN150/125. Keep Sumaya PS_400.</t>
         </is>
       </c>
-      <c r="K29" s="3" t="inlineStr">
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>محطة سمية وليس بوستر حيان (YWC + خط DN400 مباشر من سمية). يبقى Sumaya PS_400</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="N29" s="2" t="inlineStr">
         <is>
           <t>Sumaya PS_400</t>
         </is>
       </c>
-      <c r="M29" s="2" t="n">
+      <c r="O29" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2291,25 +2586,35 @@
           <t>Check if fe from Sumaya_PS or Hayyan_Booster ?</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة سمية أم بوستر حيان؟</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>Sumaya PS (not Hayyan). YWC: SUMAYYA PS. But field notes: separate DN200 direct from Sumaya PS -&gt; DN150 -&gt; DN125, not the DN400 line. Change to Sumaya PS_200.</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>محطة سمية وليس حيان، لكن من خط DN200 منفصل ← تغيير إلى Sumaya PS_200 - تأكيد</t>
+        </is>
+      </c>
+      <c r="M30" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>Sumaya PS_200</t>
         </is>
       </c>
-      <c r="M30" s="2" t="n">
+      <c r="O30" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N30" s="2" t="inlineStr">
+      <c r="P30" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2355,25 +2660,35 @@
           <t>Check from where it's fed Bwaida_Reservoir_300_gravity or Rehab_Resv ?</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>التحقق من مصدر التغذية: خط البويضة 300 بالانسياب أم خزان رحاب؟</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>Bweidha DN300 - NOT Rehab. Field: DN63/100 from DN150 on DN300 from Bweidha PS, fed from the north. YWC: HAMAMT OMOUSH / BWAIDAH PS. Rhab PS is only a 60m3/h@300m booster. Keep Bweidha_Resv_300_G.</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr">
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>من خط البويضة DN300 من الشمال وليس رحاب. YWC: حمامة العموش/البويضة. يبقى Bweidha_Resv_300_G</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>Bweidha_Resv_300_G</t>
         </is>
       </c>
-      <c r="M31" s="2" t="n">
+      <c r="O31" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2415,25 +2730,35 @@
           <t>Check if fed from Dogmseh_PS or Bweida_PS</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة الدقمسة أم محطة البويضة</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS. YWC: DOGMOSEH PS. Dogmseh PS (2 pumps 50m3/h@400m/@250m, 4x25m3 tanks) is fed from Bweidha system; zone boosted by Dogmseh PS; PS is inside this zone. Keep Dogmseh_PS.</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>محطة الدقمسة (YWC) والمحطة داخل المنطقة. يبقى Dogmseh_PS</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS</t>
         </is>
       </c>
-      <c r="M32" s="2" t="n">
+      <c r="O32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N32" s="2" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2475,25 +2800,35 @@
           <t>2 discharge pipes ? if yes split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع؟ إذا نعم تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>Yes, Zubaidiyeh PS has &gt;1 discharge: 2 pumps (50m3/h@100m, 100m3/h@150m) + DN150/DN125/DN100 outlets (field). This zone: DN100 direct from PS -&gt; Al Zubaideyeh_PS_100.</t>
         </is>
       </c>
-      <c r="K33" s="4" t="inlineStr">
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>نعم أكثر من خط دفع (مضختان وخطوط DN150/125/100). هذه المنطقة DN100 ← Al Zubaideyeh_PS_100</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>Al Zubaideyeh_PS_100</t>
         </is>
       </c>
-      <c r="M33" s="2" t="n">
+      <c r="O33" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N33" s="2" t="inlineStr">
+      <c r="P33" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2539,25 +2874,35 @@
           <t>2 discharge pipes ? if yes split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع؟ إذا نعم تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Yes, Zubaidiyeh PS has &gt;1 discharge: 2 pumps (50m3/h@100m, 100m3/h@150m) + DN150/DN125/DN100 outlets (field). This zone: DN150 from PS -&gt; Al Zubaideyeh_PS_150.</t>
         </is>
       </c>
-      <c r="K34" s="4" t="inlineStr">
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>نعم أكثر من خط دفع (مضختان وخطوط DN150/125/100). هذه المنطقة DN150 ← Al Zubaideyeh_PS_150</t>
+        </is>
+      </c>
+      <c r="M34" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>Al Zubaideyeh_PS_150</t>
         </is>
       </c>
-      <c r="M34" s="2" t="n">
+      <c r="O34" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N34" s="2" t="inlineStr">
+      <c r="P34" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2603,25 +2948,35 @@
           <t>2 discharge pipes ? if yes split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع؟ إذا نعم تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>Yes, Zubaidiyeh PS has &gt;1 discharge: 2 pumps (50m3/h@100m, 100m3/h@150m) + DN150/DN125/DN100 outlets (field). This zone: DN125 PE from PS -&gt; Al Zubaideyeh_PS_125.</t>
         </is>
       </c>
-      <c r="K35" s="4" t="inlineStr">
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>نعم أكثر من خط دفع (مضختان وخطوط DN150/125/100). هذه المنطقة DN125 ← Al Zubaideyeh_PS_125</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>Al Zubaideyeh_PS_125</t>
         </is>
       </c>
-      <c r="M35" s="2" t="n">
+      <c r="O35" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N35" s="2" t="inlineStr">
+      <c r="P35" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2667,25 +3022,35 @@
           <t>2 discharge pipes ? if yes split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع؟ إذا نعم تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>Yes, Zubaidiyeh PS has &gt;1 discharge: 2 pumps (50m3/h@100m, 100m3/h@150m) + DN150/DN125/DN100 outlets (field). This zone: DN125 from PS -&gt; Al Zubaideyeh_PS_125.</t>
         </is>
       </c>
-      <c r="K36" s="4" t="inlineStr">
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>نعم أكثر من خط دفع (مضختان وخطوط DN150/125/100). هذه المنطقة DN125 ← Al Zubaideyeh_PS_125</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr">
         <is>
           <t>Al Zubaideyeh_PS_125</t>
         </is>
       </c>
-      <c r="M36" s="2" t="n">
+      <c r="O36" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N36" s="2" t="inlineStr">
+      <c r="P36" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2731,25 +3096,35 @@
           <t>2 discharge pipes ? if yes split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع؟ إذا نعم تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>Yes, Zubaidiyeh PS has &gt;1 discharge: 2 pumps (50m3/h@100m, 100m3/h@150m) + DN150/DN125/DN100 outlets (field). This zone: DN125 from PS -&gt; Al Zubaideyeh_PS_125.</t>
         </is>
       </c>
-      <c r="K37" s="4" t="inlineStr">
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>نعم أكثر من خط دفع (مضختان وخطوط DN150/125/100). هذه المنطقة DN125 ← Al Zubaideyeh_PS_125</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
+      <c r="N37" s="2" t="inlineStr">
         <is>
           <t>Al Zubaideyeh_PS_125</t>
         </is>
       </c>
-      <c r="M37" s="2" t="n">
+      <c r="O37" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N37" s="2" t="inlineStr">
+      <c r="P37" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2795,25 +3170,35 @@
           <t>2 discharge pipes ? if yes split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع؟ إذا نعم تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>Yes, Zubaidiyeh PS has &gt;1 discharge: 2 pumps (50m3/h@100m, 100m3/h@150m) + DN150/DN125/DN100 outlets (field). This zone: DN150 from PS -&gt; Al Zubaideyeh_PS_150.</t>
         </is>
       </c>
-      <c r="K38" s="4" t="inlineStr">
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>نعم أكثر من خط دفع (مضختان وخطوط DN150/125/100). هذه المنطقة DN150 ← Al Zubaideyeh_PS_150</t>
+        </is>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr">
+      <c r="N38" s="2" t="inlineStr">
         <is>
           <t>Al Zubaideyeh_PS_150</t>
         </is>
       </c>
-      <c r="M38" s="2" t="n">
+      <c r="O38" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N38" s="2" t="inlineStr">
+      <c r="P38" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2859,25 +3244,35 @@
           <t>2 discharge pipes ? if yes split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع؟ إذا نعم تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>Yes, Zubaidiyeh PS has &gt;1 discharge: 2 pumps (50m3/h@100m, 100m3/h@150m) + DN150/DN125/DN100 outlets (field). This zone: DN100 from PS -&gt; Al Zubaideyeh_PS_100.</t>
         </is>
       </c>
-      <c r="K39" s="4" t="inlineStr">
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>نعم أكثر من خط دفع (مضختان وخطوط DN150/125/100). هذه المنطقة DN100 ← Al Zubaideyeh_PS_100</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
+      <c r="N39" s="2" t="inlineStr">
         <is>
           <t>Al Zubaideyeh_PS_100</t>
         </is>
       </c>
-      <c r="M39" s="2" t="n">
+      <c r="O39" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N39" s="2" t="inlineStr">
+      <c r="P39" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2923,25 +3318,35 @@
           <t>is there 2 discharge from the PS 100 + 150 ? PS Um-Serb PS feed  Zubeydeh PS or invers ?</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع 100 + 150 من المحطة؟ هل أم السرب تغذي الزبيدية أم العكس؟</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>Yes, 2 discharges: DN100 + DN150 (field notes; pumps 100m3/h@150m + 50m3/h@200m). Direction Um Serb&lt;-&gt;Zubaidiyeh unknown (both Zaatari WS) - ask operator. Zone on DN100 -&gt; Um EsSerb PS_100</t>
         </is>
       </c>
-      <c r="K40" s="5" t="inlineStr">
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>نعم خطا دفع DN100 وDN150. اتجاه التغذية بين أم السرب والزبيدية غير معروف - اسأل المشغل. DN100 ← Um EsSerb PS_100</t>
+        </is>
+      </c>
+      <c r="M40" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="N40" s="2" t="inlineStr">
         <is>
           <t>Um EsSerb PS_100</t>
         </is>
       </c>
-      <c r="M40" s="2" t="n">
+      <c r="O40" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N40" s="2" t="inlineStr">
+      <c r="P40" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2987,25 +3392,35 @@
           <t>is there 2 discharge from the PS 100 + 150 ? PS Um-Serb PS feed  Zubeydeh PS or invers ?</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع 100 + 150 من المحطة؟ هل أم السرب تغذي الزبيدية أم العكس؟</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>Yes, 2 discharges: DN100 + DN150 (field notes; pumps 100m3/h@150m + 50m3/h@200m). Direction Um Serb&lt;-&gt;Zubaidiyeh unknown (both Zaatari WS) - ask operator. Zone on DN150 -&gt; Um EsSerb PS_150</t>
         </is>
       </c>
-      <c r="K41" s="5" t="inlineStr">
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>نعم خطا دفع DN100 وDN150. اتجاه التغذية بين أم السرب والزبيدية غير معروف - اسأل المشغل. DN150 ← Um EsSerb PS_150</t>
+        </is>
+      </c>
+      <c r="M41" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L41" s="2" t="inlineStr">
+      <c r="N41" s="2" t="inlineStr">
         <is>
           <t>Um EsSerb PS_150</t>
         </is>
       </c>
-      <c r="M41" s="2" t="n">
+      <c r="O41" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N41" s="2" t="inlineStr">
+      <c r="P41" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3051,25 +3466,35 @@
           <t>is there 2 discharge from the PS 100 + 150 ? PS Um-Serb PS feed  Zubeydeh PS or invers ?</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع 100 + 150 من المحطة؟ هل أم السرب تغذي الزبيدية أم العكس؟</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>Yes, 2 discharges: DN100 + DN150 (field notes; pumps 100m3/h@150m + 50m3/h@200m). Direction Um Serb&lt;-&gt;Zubaidiyeh unknown (both Zaatari WS) - ask operator. Zone on separate DN100 -&gt; Um EsSerb PS_100</t>
         </is>
       </c>
-      <c r="K42" s="5" t="inlineStr">
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>نعم خطا دفع DN100 وDN150. اتجاه التغذية بين أم السرب والزبيدية غير معروف - اسأل المشغل. DN100 ← Um EsSerb PS_100</t>
+        </is>
+      </c>
+      <c r="M42" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>Um EsSerb PS_100</t>
         </is>
       </c>
-      <c r="M42" s="2" t="n">
+      <c r="O42" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N42" s="2" t="inlineStr">
+      <c r="P42" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3115,25 +3540,35 @@
           <t>is there 2 discharge from the PS 100 + 150 ? PS Um-Serb PS feed  Zubeydeh PS or invers ?</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع 100 + 150 من المحطة؟ هل أم السرب تغذي الزبيدية أم العكس؟</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>Yes, 2 discharges: DN100 + DN150 (field notes; pumps 100m3/h@150m + 50m3/h@200m). Direction Um Serb&lt;-&gt;Zubaidiyeh unknown (both Zaatari WS) - ask operator. Zone on separate DN100 -&gt; Um EsSerb PS_100</t>
         </is>
       </c>
-      <c r="K43" s="5" t="inlineStr">
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>نعم خطا دفع DN100 وDN150. اتجاه التغذية بين أم السرب والزبيدية غير معروف - اسأل المشغل. DN100 ← Um EsSerb PS_100</t>
+        </is>
+      </c>
+      <c r="M43" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr">
+      <c r="N43" s="2" t="inlineStr">
         <is>
           <t>Um EsSerb PS_100</t>
         </is>
       </c>
-      <c r="M43" s="2" t="n">
+      <c r="O43" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N43" s="2" t="inlineStr">
+      <c r="P43" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3179,25 +3614,35 @@
           <t>is there 2 discharge from the PS 100 + 150 ? PS Um-Serb PS feed  Zubeydeh PS or invers ?</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>هل يوجد خطا دفع 100 + 150 من المحطة؟ هل أم السرب تغذي الزبيدية أم العكس؟</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>Yes, 2 discharges: DN100 + DN150 (field notes; pumps 100m3/h@150m + 50m3/h@200m). Direction Um Serb&lt;-&gt;Zubaidiyeh unknown (both Zaatari WS) - ask operator. Zone on DN150 -&gt; Um EsSerb PS_150</t>
         </is>
       </c>
-      <c r="K44" s="5" t="inlineStr">
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>نعم خطا دفع DN100 وDN150. اتجاه التغذية بين أم السرب والزبيدية غير معروف - اسأل المشغل. DN150 ← Um EsSerb PS_150</t>
+        </is>
+      </c>
+      <c r="M44" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr">
+      <c r="N44" s="2" t="inlineStr">
         <is>
           <t>Um EsSerb PS_150</t>
         </is>
       </c>
-      <c r="M44" s="2" t="n">
+      <c r="O44" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N44" s="2" t="inlineStr">
+      <c r="P44" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3243,25 +3688,35 @@
           <t>check if fed by DN200 from Balaama Resv by gravity ? or from Znayah PS ?</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية بخط DN200 من خزان بلعما بالانسياب أم من محطة الزنية؟</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>Balaama Resv by gravity (DN200), not Znayah PS. YWC: 'Balaam Res (By Gravity)' for Balaama Phase 1 + Hay Al Hussein. Balaama tank 1000m3 is 220 m away (pumps only H=70m). Change to Balaama_Resv_200_G.</t>
         </is>
       </c>
-      <c r="K45" s="3" t="inlineStr">
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>خزان بلعما بالانسياب DN200 وليس الزنية (YWC). تغيير إلى Balaama_Resv_200_G</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="N45" s="2" t="inlineStr">
         <is>
           <t>Balaama_Resv_200_G</t>
         </is>
       </c>
-      <c r="M45" s="2" t="n">
+      <c r="O45" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N45" s="2" t="inlineStr">
+      <c r="P45" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3307,25 +3762,35 @@
           <t>check if fed by DN200 from Balaama Resv by gravity ? or from Znayah PS_DN200 ?</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية بخط DN200 من خزان بلعما بالانسياب أم من محطة الزنية؟</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>Mixed - split polygon: Hay Aggad = Balaama Resv gravity (YWC 62%), Balaama Hay Shamali = Znayah PS (YWC 33%). Field: DN200 from PS with DN125 branches. Keep Znayah_PS_200 for north part; confirm split line.</t>
         </is>
       </c>
-      <c r="K46" s="4" t="inlineStr">
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>مختلطة - تقسيم: حي العقاد من خزان بلعما بالانسياب، وبلعما الحي الشمالي من محطة الزنية DN200. تأكيد</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="N46" s="2" t="inlineStr">
         <is>
           <t>Znayah_PS_200 + Balaama_Resv_200_G</t>
         </is>
       </c>
-      <c r="M46" s="2" t="n">
+      <c r="O46" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N46" s="2" t="inlineStr">
+      <c r="P46" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3371,25 +3836,35 @@
           <t>check if fed by DN200 from Balaama Resv by gravity ? or from Znayah PS_DN200 ?</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية بخط DN200 من خزان بلعما بالانسياب أم من محطة الزنية؟</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>Znayah PS DN200 (not Balaama gravity). YWC: MORTAFAAT BALAAMA / Znayyah PS; high area; field: DN100 from DN200 from PS. Keep Znayah_PS_200.</t>
         </is>
       </c>
-      <c r="K47" s="3" t="inlineStr">
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>محطة الزنية DN200 وليس انسياب بلعما (YWC، منطقة مرتفعة). يبقى Znayah_PS_200</t>
+        </is>
+      </c>
+      <c r="M47" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L47" s="2" t="inlineStr">
+      <c r="N47" s="2" t="inlineStr">
         <is>
           <t>Znayah_PS_200</t>
         </is>
       </c>
-      <c r="M47" s="2" t="n">
+      <c r="O47" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N47" s="2" t="inlineStr"/>
+      <c r="P47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -3431,25 +3906,35 @@
           <t>Check if really from Baaj_PS_2 ? how many discharge lines ? if more then 1 split the hydraulic zone.</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً من محطة الباعج 2؟ كم خط دفع؟ إذا أكثر من خط يتم التقسيم</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>Yes, BAEJ 2 PS (YWC confirms, 2 pumps 100m3/h@150m). 2 outlets DN150 + DN100 -&gt; split. This zone: DN150 direct -&gt; BAEJ 2_PS_150.</t>
         </is>
       </c>
-      <c r="K48" s="4" t="inlineStr">
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>نعم من الباعج 2 (YWC). خطا دفع DN150 وDN100 ← تقسيم. هذه المنطقة ← BAEJ 2_PS_150</t>
+        </is>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L48" s="2" t="inlineStr">
+      <c r="N48" s="2" t="inlineStr">
         <is>
           <t>BAEJ 2_PS_150</t>
         </is>
       </c>
-      <c r="M48" s="2" t="n">
+      <c r="O48" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N48" s="2" t="inlineStr">
+      <c r="P48" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3495,25 +3980,35 @@
           <t>Check if really from Baaj_PS_2 ? how many discharge lines ? if more then 1 split the hydraulic zone.</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr">
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً من محطة الباعج 2؟ كم خط دفع؟ إذا أكثر من خط يتم التقسيم</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>Yes, BAEJ 2 PS (YWC confirms, 2 pumps 100m3/h@150m). 2 outlets DN150 + DN100 -&gt; split. This zone: DN100-&gt;50 direct -&gt; BAEJ 2_PS_100.</t>
         </is>
       </c>
-      <c r="K49" s="4" t="inlineStr">
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>نعم من الباعج 2 (YWC). خطا دفع DN150 وDN100 ← تقسيم. هذه المنطقة ← BAEJ 2_PS_100</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L49" s="2" t="inlineStr">
+      <c r="N49" s="2" t="inlineStr">
         <is>
           <t>BAEJ 2_PS_100</t>
         </is>
       </c>
-      <c r="M49" s="2" t="n">
+      <c r="O49" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N49" s="2" t="inlineStr">
+      <c r="P49" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3559,25 +4054,35 @@
           <t>Check if really from Baaj_PS_2 ? how many discharge lines ? if more then 1 split the hydraulic zone.</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً من محطة الباعج 2؟ كم خط دفع؟ إذا أكثر من خط يتم التقسيم</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>Yes, BAEJ 2 PS (YWC confirms, 2 pumps 100m3/h@150m). 2 outlets DN150 + DN100 -&gt; split. This zone: DN100 -&gt; BAEJ 2_PS_100.</t>
         </is>
       </c>
-      <c r="K50" s="4" t="inlineStr">
+      <c r="L50" s="3" t="inlineStr">
+        <is>
+          <t>نعم من الباعج 2 (YWC). خطا دفع DN150 وDN100 ← تقسيم. هذه المنطقة ← BAEJ 2_PS_100</t>
+        </is>
+      </c>
+      <c r="M50" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L50" s="2" t="inlineStr">
+      <c r="N50" s="2" t="inlineStr">
         <is>
           <t>BAEJ 2_PS_100</t>
         </is>
       </c>
-      <c r="M50" s="2" t="n">
+      <c r="O50" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N50" s="2" t="inlineStr">
+      <c r="P50" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3623,25 +4128,35 @@
           <t>Check if really from Baaj_PS_2 ? how many discharge lines ? if more then 1 split the hydraulic zone.</t>
         </is>
       </c>
-      <c r="J51" s="2" t="inlineStr">
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً من محطة الباعج 2؟ كم خط دفع؟ إذا أكثر من خط يتم التقسيم</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
         <is>
           <t>Yes, BAEJ 2 PS (YWC confirms, 2 pumps 100m3/h@150m). 2 outlets DN150 + DN100 -&gt; split. This zone: collector valve DN50/25 -&gt; BAEJ 2_PS_100 (confirm which outlet).</t>
         </is>
       </c>
-      <c r="K51" s="4" t="inlineStr">
+      <c r="L51" s="3" t="inlineStr">
+        <is>
+          <t>نعم من الباعج 2 (YWC). خطا دفع DN150 وDN100 ← تقسيم. هذه المنطقة ← BAEJ 2_PS_100</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L51" s="2" t="inlineStr">
+      <c r="N51" s="2" t="inlineStr">
         <is>
           <t>BAEJ 2_PS_100</t>
         </is>
       </c>
-      <c r="M51" s="2" t="n">
+      <c r="O51" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N51" s="2" t="inlineStr">
+      <c r="P51" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3687,25 +4202,35 @@
           <t>Check if really from Baaj_PS_2 ? how many discharge lines ? if more then 1 split the hydraulic zone.</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل فعلاً من محطة الباعج 2؟ كم خط دفع؟ إذا أكثر من خط يتم التقسيم</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
         <is>
           <t>Yes, BAEJ 2 PS (YWC confirms, 2 pumps 100m3/h@150m). 2 outlets DN150 + DN100 -&gt; split. This zone: main line + DN100 to Mebrek -&gt; BAEJ 2_PS_100.</t>
         </is>
       </c>
-      <c r="K52" s="4" t="inlineStr">
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>نعم من الباعج 2 (YWC). خطا دفع DN150 وDN100 ← تقسيم. هذه المنطقة ← BAEJ 2_PS_100</t>
+        </is>
+      </c>
+      <c r="M52" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L52" s="2" t="inlineStr">
+      <c r="N52" s="2" t="inlineStr">
         <is>
           <t>BAEJ 2_PS_100</t>
         </is>
       </c>
-      <c r="M52" s="2" t="n">
+      <c r="O52" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N52" s="2" t="inlineStr">
+      <c r="P52" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3751,25 +4276,35 @@
           <t>To check with operator if realy from Baaj PS 3 ? how many discharge ?</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr">
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>التحقق مع المشغل هل فعلاً من محطة الباعج 3؟ كم خط دفع؟</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
         <is>
           <t>Yes, BAEJ 3 PS (YWC confirms; PS inside zone 459). 1 pump 50m3/h@100m, outlets are DN100 from the same collector = same head -&gt; no split needed.</t>
         </is>
       </c>
-      <c r="K53" s="3" t="inlineStr">
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>نعم من الباعج 3 (YWC). مضخة واحدة وخطوط DN100 من نفس المجمع ← لا حاجة للتقسيم</t>
+        </is>
+      </c>
+      <c r="M53" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L53" s="2" t="inlineStr">
+      <c r="N53" s="2" t="inlineStr">
         <is>
           <t>BAEJ 3_PS</t>
         </is>
       </c>
-      <c r="M53" s="2" t="n">
+      <c r="O53" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N53" s="2" t="inlineStr"/>
+      <c r="P53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -3811,25 +4346,35 @@
           <t>To check with operator if realy from Baaj PS 3 ? how many discharge ?</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>التحقق مع المشغل هل فعلاً من محطة الباعج 3؟ كم خط دفع؟</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
         <is>
           <t>Yes, BAEJ 3 PS (YWC confirms; PS inside zone 459). 1 pump 50m3/h@100m, outlets are DN100 from the same collector = same head -&gt; no split needed.</t>
         </is>
       </c>
-      <c r="K54" s="3" t="inlineStr">
+      <c r="L54" s="3" t="inlineStr">
+        <is>
+          <t>نعم من الباعج 3 (YWC). مضخة واحدة وخطوط DN100 من نفس المجمع ← لا حاجة للتقسيم</t>
+        </is>
+      </c>
+      <c r="M54" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr">
+      <c r="N54" s="2" t="inlineStr">
         <is>
           <t>BAEJ 3_PS</t>
         </is>
       </c>
-      <c r="M54" s="2" t="n">
+      <c r="O54" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N54" s="2" t="inlineStr"/>
+      <c r="P54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -3871,25 +4416,35 @@
           <t>Fed by Hosha booster ? or um Lulu ps ?</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>هل التغذية من بوستر حوشا أم من محطة أم اللولو؟</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
         <is>
           <t>Hosha Booster (not Um Lulu PS pumps). Um Lulu Resv feeds the booster by gravity DN200, booster (2 pumps) feeds zone. YWC: 'UM LOLO GRAVITY TO BOOSTER HOSHA'. Hosha Resv abandoned. Keep Hosha_Booster_150.</t>
         </is>
       </c>
-      <c r="K55" s="3" t="inlineStr">
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>بوستر حوشا وليس مضخات أم اللولو: خزان أم اللولو يغذي البوستر بالانسياب DN200. يبقى Hosha_Booster_150</t>
+        </is>
+      </c>
+      <c r="M55" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L55" s="2" t="inlineStr">
+      <c r="N55" s="2" t="inlineStr">
         <is>
           <t>Hosha_Booster_150</t>
         </is>
       </c>
-      <c r="M55" s="2" t="n">
+      <c r="O55" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N55" s="2" t="inlineStr"/>
+      <c r="P55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -3931,25 +4486,35 @@
           <t>check if fed by DN200 from Balaama Resv by gravity ? or from Znayah PS_DN200 ?</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr">
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية بخط DN200 من خزان بلعما بالانسياب أم من محطة الزنية؟</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
         <is>
           <t>Znayah PS (not Balaama gravity). YWC: HAMNANAH+BOSTANAH+UM SWEINEH / Znayyah PS. Field: DN180 + DN300 from PS -&gt; may be Znayah_PS_300_1 rather than _200; confirm which line.</t>
         </is>
       </c>
-      <c r="K56" s="4" t="inlineStr">
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>محطة الزنية (YWC)، لكن التغذية من خطي 180 و300 ← ربما Znayah_PS_300_1 - تأكيد</t>
+        </is>
+      </c>
+      <c r="M56" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L56" s="2" t="inlineStr">
+      <c r="N56" s="2" t="inlineStr">
         <is>
           <t>Znayah_PS_300_1</t>
         </is>
       </c>
-      <c r="M56" s="2" t="n">
+      <c r="O56" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N56" s="2" t="inlineStr">
+      <c r="P56" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3995,25 +4560,35 @@
           <t>To check P_Zone : Balela Reservoir instead of Bowidah_PS</t>
         </is>
       </c>
-      <c r="J57" s="2" t="inlineStr">
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>التحقق من منطقة الضغط: خزان بليلا بدلاً من محطة البويضة</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
         <is>
           <t>Yes - change to Balela Resv (gravity). Bowidah PS pumps to Balela Resv; field: gravity DN100 from DN150 from Balela Resv. Change to Balela_Resv (not in YWC Mafraq layer).</t>
         </is>
       </c>
-      <c r="K57" s="3" t="inlineStr">
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>نعم تغيير إلى Balela_Resv: محطة البويضة تضخ لخزان بليلا والمنطقة تتغذى منه بالانسياب</t>
+        </is>
+      </c>
+      <c r="M57" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L57" s="2" t="inlineStr">
+      <c r="N57" s="2" t="inlineStr">
         <is>
           <t>Balela_Resv</t>
         </is>
       </c>
-      <c r="M57" s="2" t="n">
+      <c r="O57" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N57" s="2" t="inlineStr">
+      <c r="P57" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4059,25 +4634,35 @@
           <t>Fed by Hosha booster or Um Lulu PS ?</t>
         </is>
       </c>
-      <c r="J58" s="2" t="inlineStr">
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>هل التغذية من بوستر حوشا أم من محطة أم اللولو؟</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
         <is>
           <t>Hosha Booster (not Um Lulu PS pumps). Um Lulu Resv feeds the booster by gravity DN200, booster DN200 discharge feeds Bwaidha. YWC: 'UM LOLO GRAVITY TO HOSHA BOOSTER'. Keep Hosha_Booster_200.</t>
         </is>
       </c>
-      <c r="K58" s="3" t="inlineStr">
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>بوستر حوشا وليس مضخات أم اللولو: خزان أم اللولو يغذي البوستر بالانسياب DN200. يبقى Hosha_Booster_200</t>
+        </is>
+      </c>
+      <c r="M58" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L58" s="2" t="inlineStr">
+      <c r="N58" s="2" t="inlineStr">
         <is>
           <t>Hosha_Booster_200</t>
         </is>
       </c>
-      <c r="M58" s="2" t="n">
+      <c r="O58" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N58" s="2" t="inlineStr"/>
+      <c r="P58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -4119,25 +4704,35 @@
           <t>Fed by Hosha booster or Um Lulu PS ?</t>
         </is>
       </c>
-      <c r="J59" s="2" t="inlineStr">
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>هل التغذية من بوستر حوشا أم من محطة أم اللولو؟</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
         <is>
           <t>Hosha Booster (not Um Lulu PS pumps). Um Lulu Resv feeds the booster by gravity DN200, booster DN200 discharge feeds Bwaidha. YWC: 'UM LOLO GRAVITY TO HOSHA BOOSTER'. Keep Hosha_Booster_200.</t>
         </is>
       </c>
-      <c r="K59" s="3" t="inlineStr">
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>بوستر حوشا وليس مضخات أم اللولو: خزان أم اللولو يغذي البوستر بالانسياب DN200. يبقى Hosha_Booster_200</t>
+        </is>
+      </c>
+      <c r="M59" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L59" s="2" t="inlineStr">
+      <c r="N59" s="2" t="inlineStr">
         <is>
           <t>Hosha_Booster_200</t>
         </is>
       </c>
-      <c r="M59" s="2" t="n">
+      <c r="O59" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N59" s="2" t="inlineStr"/>
+      <c r="P59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -4179,25 +4774,35 @@
           <t>Fed by Hosha booster or Um Lulu PS ?</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr">
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>هل التغذية من بوستر حوشا أم من محطة أم اللولو؟</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
         <is>
           <t>Hosha Booster (not Um Lulu PS pumps). Um Lulu Resv feeds the booster by gravity DN200, booster DN200 discharge feeds Bwaidha. YWC: 'UM LOLO GRAVITY TO HOSHA BOOSTER'. Keep Hosha_Booster_200.</t>
         </is>
       </c>
-      <c r="K60" s="3" t="inlineStr">
+      <c r="L60" s="3" t="inlineStr">
+        <is>
+          <t>بوستر حوشا وليس مضخات أم اللولو: خزان أم اللولو يغذي البوستر بالانسياب DN200. يبقى Hosha_Booster_200</t>
+        </is>
+      </c>
+      <c r="M60" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L60" s="2" t="inlineStr">
+      <c r="N60" s="2" t="inlineStr">
         <is>
           <t>Hosha_Booster_200</t>
         </is>
       </c>
-      <c r="M60" s="2" t="n">
+      <c r="O60" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N60" s="2" t="inlineStr"/>
+      <c r="P60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -4239,25 +4844,35 @@
           <t>Fed by Hosha booster or Um Lulu PS ?</t>
         </is>
       </c>
-      <c r="J61" s="2" t="inlineStr">
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>هل التغذية من بوستر حوشا أم من محطة أم اللولو؟</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
         <is>
           <t>Hosha Booster (not Um Lulu PS pumps). Um Lulu Resv feeds the booster by gravity DN200, booster DN200 discharge feeds Bwaidha. YWC: 'UM LOLO GRAVITY TO HOSHA BOOSTER'. Keep Hosha_Booster_200.</t>
         </is>
       </c>
-      <c r="K61" s="3" t="inlineStr">
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>بوستر حوشا وليس مضخات أم اللولو: خزان أم اللولو يغذي البوستر بالانسياب DN200. يبقى Hosha_Booster_200</t>
+        </is>
+      </c>
+      <c r="M61" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L61" s="2" t="inlineStr">
+      <c r="N61" s="2" t="inlineStr">
         <is>
           <t>Hosha_Booster_200</t>
         </is>
       </c>
-      <c r="M61" s="2" t="n">
+      <c r="O61" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N61" s="2" t="inlineStr"/>
+      <c r="P61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -4299,25 +4914,35 @@
           <t>Fed by Hosha booster or Um Lulu PS ?</t>
         </is>
       </c>
-      <c r="J62" s="2" t="inlineStr">
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>هل التغذية من بوستر حوشا أم من محطة أم اللولو؟</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
         <is>
           <t>Hosha Booster (not Um Lulu PS pumps). Um Lulu Resv feeds the booster by gravity DN200, booster DN200 discharge feeds Bwaidha. YWC: 'UM LOLO GRAVITY TO HOSHA BOOSTER'. Keep Hosha_Booster_200.</t>
         </is>
       </c>
-      <c r="K62" s="3" t="inlineStr">
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>بوستر حوشا وليس مضخات أم اللولو: خزان أم اللولو يغذي البوستر بالانسياب DN200. يبقى Hosha_Booster_200</t>
+        </is>
+      </c>
+      <c r="M62" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L62" s="2" t="inlineStr">
+      <c r="N62" s="2" t="inlineStr">
         <is>
           <t>Hosha_Booster_200</t>
         </is>
       </c>
-      <c r="M62" s="2" t="n">
+      <c r="O62" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N62" s="2" t="inlineStr"/>
+      <c r="P62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -4359,25 +4984,35 @@
           <t>Check if fed from Dogmseh_PS or Bweida_PS</t>
         </is>
       </c>
-      <c r="J63" s="2" t="inlineStr">
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة الدقمسة أم محطة البويضة</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS. YWC: DOGMOSEH PS. Dogmseh PS (2 pumps 50m3/h@400m/@250m, 4x25m3 tanks) is fed from Bweidha system; zone boosted by Dogmseh PS, 4 sub-zones 6h each. Keep Dogmseh_PS.</t>
         </is>
       </c>
-      <c r="K63" s="3" t="inlineStr">
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>محطة الدقمسة (YWC)، 4 مناطق فرعية 6 ساعات لكل منها. يبقى Dogmseh_PS</t>
+        </is>
+      </c>
+      <c r="M63" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L63" s="2" t="inlineStr">
+      <c r="N63" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS</t>
         </is>
       </c>
-      <c r="M63" s="2" t="n">
+      <c r="O63" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N63" s="2" t="inlineStr"/>
+      <c r="P63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -4419,25 +5054,35 @@
           <t>Check if fed from Dogmseh_PS or Bweida_PS</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr">
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة الدقمسة أم محطة البويضة</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS (boosted from SP Dogmosseh - field; Dogmseh 4 km vs Bweidha PS 11 km). YWC lists BWAIDAH PS = origin of water feeding Dogmseh. Keep Dogmseh_PS; confirm booster runs every cycle.</t>
         </is>
       </c>
-      <c r="K64" s="4" t="inlineStr">
+      <c r="L64" s="3" t="inlineStr">
+        <is>
+          <t>محطة الدقمسة (تقوية حسب الملاحظات وأقرب من البويضة). YWC يذكر البويضة كمصدر المياه. يبقى Dogmseh_PS - تأكيد</t>
+        </is>
+      </c>
+      <c r="M64" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L64" s="2" t="inlineStr">
+      <c r="N64" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS</t>
         </is>
       </c>
-      <c r="M64" s="2" t="n">
+      <c r="O64" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N64" s="2" t="inlineStr"/>
+      <c r="P64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -4479,25 +5124,35 @@
           <t>Check if fed from Dogmseh_PS or Bweida_PS</t>
         </is>
       </c>
-      <c r="J65" s="2" t="inlineStr">
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>التحقق هل التغذية من محطة الدقمسة أم محطة البويضة</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS (boosted from SP Dogmosseh - field; Dogmseh 5 km vs Bweidha PS 13 km). YWC lists BWAIDAH PS = origin of water feeding Dogmseh. Keep Dogmseh_PS; confirm booster runs every cycle.</t>
         </is>
       </c>
-      <c r="K65" s="4" t="inlineStr">
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>محطة الدقمسة (تقوية حسب الملاحظات وأقرب من البويضة). YWC يذكر البويضة كمصدر المياه. يبقى Dogmseh_PS - تأكيد</t>
+        </is>
+      </c>
+      <c r="M65" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L65" s="2" t="inlineStr">
+      <c r="N65" s="2" t="inlineStr">
         <is>
           <t>Dogmseh_PS</t>
         </is>
       </c>
-      <c r="M65" s="2" t="n">
+      <c r="O65" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N65" s="2" t="inlineStr"/>
+      <c r="P65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -4539,25 +5194,35 @@
           <t>How many discharge lines ? split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J66" s="2" t="inlineStr">
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>كم عدد خطوط الدفع؟ تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>Koum Ahmar PS has 2 pumps (50m3/h@250m, 100m3/h@100m) and 2 distribution outlets DN125 + DN100 (field notes). This zone fed by DN100 -&gt; Koum Ahmar_PS_100. Confirm which pump feeds which line.</t>
         </is>
       </c>
-      <c r="K66" s="4" t="inlineStr">
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>لمحطة الكوم الأحمر خطا توزيع DN125 وDN100. هذه المنطقة على DN100 ← Koum Ahmar_PS_100 - تأكيد مع المشغل</t>
+        </is>
+      </c>
+      <c r="M66" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L66" s="2" t="inlineStr">
+      <c r="N66" s="2" t="inlineStr">
         <is>
           <t>Koum Ahmar_PS_100</t>
         </is>
       </c>
-      <c r="M66" s="2" t="n">
+      <c r="O66" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N66" s="2" t="inlineStr">
+      <c r="P66" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4603,25 +5268,35 @@
           <t>Fed by Hosha booster or Um Lulu PS ?</t>
         </is>
       </c>
-      <c r="J67" s="2" t="inlineStr">
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>هل التغذية من بوستر حوشا أم من محطة أم اللولو؟</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
         <is>
           <t>Hosha Booster (not Um Lulu PS pumps). Um Lulu Resv feeds the booster by gravity DN200, booster DN200 discharge feeds Bwaidha. YWC: 'UM LOLO GRAVITY TO HOSHA BOOSTER'. Keep Hosha_Booster_200.</t>
         </is>
       </c>
-      <c r="K67" s="3" t="inlineStr">
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>بوستر حوشا وليس مضخات أم اللولو: خزان أم اللولو يغذي البوستر بالانسياب DN200. يبقى Hosha_Booster_200</t>
+        </is>
+      </c>
+      <c r="M67" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L67" s="2" t="inlineStr">
+      <c r="N67" s="2" t="inlineStr">
         <is>
           <t>Hosha_Booster_200</t>
         </is>
       </c>
-      <c r="M67" s="2" t="n">
+      <c r="O67" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N67" s="2" t="inlineStr"/>
+      <c r="P67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -4663,25 +5338,35 @@
           <t>To check P_Zone : Balela Reservoir instead of Bowidah_PS</t>
         </is>
       </c>
-      <c r="J68" s="2" t="inlineStr">
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>التحقق من منطقة الضغط: خزان بليلا بدلاً من محطة البويضة</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
         <is>
           <t>Yes - change to Balela Resv (gravity). Bowidah PS pumps to Balela Resv; field: DN150 feeds zone (neighbours fed from Balela Resv). Change to Balela_Resv - confirm the DN150 is the Resv outlet.</t>
         </is>
       </c>
-      <c r="K68" s="4" t="inlineStr">
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>نعم تغيير إلى Balela_Resv: محطة البويضة تضخ لخزان بليلا والمنطقة تتغذى منه بالانسياب - تأكيد</t>
+        </is>
+      </c>
+      <c r="M68" s="5" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="L68" s="2" t="inlineStr">
+      <c r="N68" s="2" t="inlineStr">
         <is>
           <t>Balela_Resv</t>
         </is>
       </c>
-      <c r="M68" s="2" t="n">
+      <c r="O68" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N68" s="2" t="inlineStr">
+      <c r="P68" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4727,25 +5412,35 @@
           <t>How many discharge lines ? split the hydraulic zone</t>
         </is>
       </c>
-      <c r="J69" s="2" t="inlineStr">
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>كم عدد خطوط الدفع؟ تقسيم المنطقة الهيدروليكية</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
         <is>
           <t>Fed from Koum Ahmar PS (YWC 58% TAREEQ KOUM AHMAR, Badia system, ROU Mafraq). Line diameter not in notes -&gt; ask operator: DN100 or DN125 outlet (Koum Ahmar_PS_100 / _125).</t>
         </is>
       </c>
-      <c r="K69" s="5" t="inlineStr">
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>من محطة الكوم الأحمر (نظام البادية). قطر الخط غير معروف - اسأل المشغل: DN100 أم DN125</t>
+        </is>
+      </c>
+      <c r="M69" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L69" s="2" t="inlineStr">
+      <c r="N69" s="2" t="inlineStr">
         <is>
           <t>Koum Ahmar_PS_100</t>
         </is>
       </c>
-      <c r="M69" s="2" t="n">
+      <c r="O69" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N69" s="2" t="inlineStr">
+      <c r="P69" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4791,32 +5486,42 @@
           <t>To check P_Zone : Balela Reservoir instead of Bowidah_PS</t>
         </is>
       </c>
-      <c r="J70" s="2" t="inlineStr">
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>التحقق من منطقة الضغط: خزان بليلا بدلاً من محطة البويضة</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
         <is>
           <t>Yes - change to Balela Resv (gravity). Bowidah PS pumps to Balela Resv; field: fed from Balela Reservoir. Change to Balela_Resv (not in YWC Mafraq layer).</t>
         </is>
       </c>
-      <c r="K70" s="3" t="inlineStr">
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>نعم تغيير إلى Balela_Resv: محطة البويضة تضخ لخزان بليلا والمنطقة تتغذى منه بالانسياب</t>
+        </is>
+      </c>
+      <c r="M70" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L70" s="2" t="inlineStr">
+      <c r="N70" s="2" t="inlineStr">
         <is>
           <t>Balela_Resv</t>
         </is>
       </c>
-      <c r="M70" s="2" t="n">
+      <c r="O70" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N70" s="2" t="inlineStr">
+      <c r="P70" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N70"/>
+  <autoFilter ref="A1:P70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>